<commit_message>
Best models validations and ML plots custom
</commit_message>
<xml_diff>
--- a/data/out/best_models_lstm/in/best_models_lstm.xlsx
+++ b/data/out/best_models_lstm/in/best_models_lstm.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\Camilo\Dev\maestria-trabajo-integrador\data\out\best_models_lstm\in\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{469048CE-F3FD-4161-86C4-A1837731AA71}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{72A6560C-1FD8-40C5-87D6-9575ECC51EE1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="24240" windowHeight="13020" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="92" uniqueCount="39">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="93" uniqueCount="40">
   <si>
     <t>variant</t>
   </si>
@@ -142,6 +142,9 @@
   </si>
   <si>
     <t>v10_date_range_no_solar_lags</t>
+  </si>
+  <si>
+    <t>config</t>
   </si>
 </sst>
 </file>
@@ -469,6 +472,9 @@
       <c r="B1" t="s">
         <v>1</v>
       </c>
+      <c r="C1" t="s">
+        <v>39</v>
+      </c>
       <c r="D1" t="s">
         <v>2</v>
       </c>

</xml_diff>